<commit_message>
fix(build): resolve duplicate import and breadcrumb prop mismatch
- Remove duplicate `getStorage` import in firebase/admin.ts
- Fix DiBreadcrumbs prop name from `items` to `segments` to match all callers

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/samples/Sample_Maintenance_BOM.xlsx
+++ b/public/samples/Sample_Maintenance_BOM.xlsx
@@ -8,9 +8,10 @@
     <sheet name="Duplicate Parts" sheetId="3" r:id="rId3"/>
     <sheet name="Missing Fields" sheetId="4" r:id="rId4"/>
     <sheet name="Revision Conflicts" sheetId="5" r:id="rId5"/>
-    <sheet name="Source Map" sheetId="6" r:id="rId6"/>
-    <sheet name="Processing Summary" sheetId="7" r:id="rId7"/>
-    <sheet name="Generic ERP Import Template" sheetId="8" r:id="rId8"/>
+    <sheet name="Low Confidence" sheetId="6" r:id="rId6"/>
+    <sheet name="Source Map" sheetId="7" r:id="rId7"/>
+    <sheet name="Processing Summary" sheetId="8" r:id="rId8"/>
+    <sheet name="Generic ERP Import Template" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Clean BOM'!A1:M8</definedName>
@@ -18,8 +19,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Duplicate Parts'!A1:I5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Missing Fields'!A1:E5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Revision Conflicts'!A1:F2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Source Map'!A1:F16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7">'Generic ERP Import Template'!A1:K1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Low Confidence'!A1:G3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Source Map'!A1:F16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8">'Generic ERP Import Template'!A1:K1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1412,6 +1414,96 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G3"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Part Number</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Confidence</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Source Page</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Validation Flags</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Recommended Action</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="B2" t="str">
+        <v>05678</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Coupling, Flexible, Jaw Type, L090</v>
+      </c>
+      <c r="D2">
+        <v>0.45</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2" t="str">
+        <v>low_confidence</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Visually verify against source document</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>15</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>Unidentified Component — Motor Mount Bracket</v>
+      </c>
+      <c r="D3">
+        <v>0.61</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3" t="str">
+        <v>missing_part_number; missing_manufacturer</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Visually verify against source document</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F16"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
@@ -1750,7 +1842,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B20"/>
   <cols>
@@ -1875,7 +1967,7 @@
         <v>Generated At</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-07-14T19:02:09.073Z</v>
+        <v>2026-07-14T21:10:05.366Z</v>
       </c>
     </row>
     <row r="17">
@@ -1905,7 +1997,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K1"/>
   <cols>

</xml_diff>